<commit_message>
Even more locked in accruals changes
</commit_message>
<xml_diff>
--- a/data/stx_xlsx/SSABa.ST.xlsx
+++ b/data/stx_xlsx/SSABa.ST.xlsx
@@ -14465,12 +14465,30 @@
       <c r="Q56" s="15">
         <v>10195.83</v>
       </c>
-      <c r="R56" s="15"/>
-      <c r="S56" s="15"/>
-      <c r="T56" s="15"/>
-      <c r="U56" s="15"/>
-      <c r="V56" s="15"/>
-      <c r="W56" s="15"/>
+      <c r="R56" s="15">
+        <f t="shared" ref="R56:W56" si="1">SUM(R58,R62,R66,R69,R72,R77)</f>
+        <v>13865.75</v>
+      </c>
+      <c r="S56" s="15">
+        <f t="shared" si="1"/>
+        <v>15637.04</v>
+      </c>
+      <c r="T56" s="15">
+        <f t="shared" si="1"/>
+        <v>17962.06</v>
+      </c>
+      <c r="U56" s="15">
+        <f t="shared" si="1"/>
+        <v>7250.5</v>
+      </c>
+      <c r="V56" s="15">
+        <f t="shared" si="1"/>
+        <v>6496.91</v>
+      </c>
+      <c r="W56" s="15">
+        <f t="shared" si="1"/>
+        <v>7086.94</v>
+      </c>
     </row>
     <row r="57" ht="15.0" customHeight="1">
       <c r="A57" s="14" t="s">

</xml_diff>